<commit_message>
Add 123 source-reviewed public academic profiles with explicit uncertainty and verified recovery build
</commit_message>
<xml_diff>
--- a/site/exports/bit-math-statistics.xlsx
+++ b/site/exports/bit-math-statistics.xlsx
@@ -14,11 +14,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'总览'!$A$1:$K$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'经历'!$A$1:$S$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'总览'!$A$1:$K$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'经历'!$A$1:$S$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'导师'!$A$1:$L$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'论文'!$A$1:$L$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'来源'!$A$1:$G$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'来源'!$A$1:$G$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -453,8 +453,8 @@
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="65" customWidth="1" min="6" max="6"/>
     <col width="37.8" customWidth="1" min="7" max="7"/>
-    <col width="26.6" customWidth="1" min="8" max="8"/>
-    <col width="21" customWidth="1" min="9" max="9"/>
+    <col width="40.59999999999999" customWidth="1" min="8" max="8"/>
+    <col width="23.8" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
   </cols>
@@ -477,7 +477,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>官方主页</t>
+          <t>个人主页／职业网站（来源类型见说明）</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -487,7 +487,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>缺项与冲突</t>
+          <t>来源说明与待核事项</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -502,7 +502,7 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>替代官方职业报道（非个人主页）</t>
+          <t>替代职业资料来源（非已核个人主页）</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
@@ -569,10 +569,64 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>吕珍涛</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>校区未标注</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>数学与统计学院</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>https://qiushi.bit.edu.cn/szdw/dsdw/xyds/2023j1/687837de84704db9853f648c9febdf0c.htm</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>未知（来源日期异常）</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Independent directory and current employment unverified; this official biography supports partial professional facts only.；No named individual works retained; zero publications means only this batch has no item-level bibliography, not that the person has no works.；No own mentor names in retained excerpts; no mentor relation inferred from own supervisor title.；Degree awards and conferral dates remain unknown unless explicitly stated.；来源记载职业信息：职业职称：预聘助理教授。上述为留存来源职业表述，不作本轮当前任职或资格认证；指导他人的资格不新增本人导师关系。</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>分批核实资料，不是完整名录；人物整体核验日期未单独记录</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>官方资料（原来源）；公开个人页（访问与内容时效见来源记录）</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>bit</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>北京理工大学</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K2"/>
+  <autoFilter ref="A1:K3"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -584,11 +638,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S8"/>
+  <dimension ref="A1:S13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="16.8" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
@@ -666,7 +720,7 @@
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>确证授位</t>
+          <t>来源记载学位</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
@@ -1140,8 +1194,293 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>吕珍涛</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>education_background</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>本科</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>北京大学</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr"/>
+      <c r="G9" s="2" t="inlineStr"/>
+      <c r="H9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="inlineStr"/>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr"/>
+      <c r="M9" s="2" t="inlineStr"/>
+      <c r="N9" s="2" t="inlineStr"/>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>本轮按留存来源记录整理；学位资格为来源记载，不代表独立证书认证。</t>
+        </is>
+      </c>
+      <c r="P9" s="2" t="inlineStr"/>
+      <c r="Q9" s="3" t="inlineStr">
+        <is>
+          <t>https://qiushi.bit.edu.cn/szdw/dsdw/xyds/2023j1/687837de84704db9853f648c9febdf0c.htm</t>
+        </is>
+      </c>
+      <c r="R9" s="2" t="inlineStr">
+        <is>
+          <t>bit</t>
+        </is>
+      </c>
+      <c r="S9" s="2" t="inlineStr">
+        <is>
+          <t>北京理工大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>吕珍涛</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>education_background</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>博士</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>宾夕法尼亚大学</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr"/>
+      <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="inlineStr"/>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr"/>
+      <c r="M10" s="2" t="inlineStr"/>
+      <c r="N10" s="2" t="inlineStr"/>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>本轮按留存来源记录整理；学位资格为来源记载，不代表独立证书认证。；来源unit：数学系</t>
+        </is>
+      </c>
+      <c r="P10" s="2" t="inlineStr"/>
+      <c r="Q10" s="3" t="inlineStr">
+        <is>
+          <t>https://qiushi.bit.edu.cn/szdw/dsdw/xyds/2023j1/687837de84704db9853f648c9febdf0c.htm</t>
+        </is>
+      </c>
+      <c r="R10" s="2" t="inlineStr">
+        <is>
+          <t>bit</t>
+        </is>
+      </c>
+      <c r="S10" s="2" t="inlineStr">
+        <is>
+          <t>北京理工大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>吕珍涛</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>education_background</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>博士后研究</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>牛津大学</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr"/>
+      <c r="G11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr"/>
+      <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="M11" s="2" t="inlineStr"/>
+      <c r="N11" s="2" t="inlineStr"/>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>本轮按留存来源记录整理；学位资格为来源记载，不代表独立证书认证。</t>
+        </is>
+      </c>
+      <c r="P11" s="2" t="inlineStr"/>
+      <c r="Q11" s="3" t="inlineStr">
+        <is>
+          <t>https://qiushi.bit.edu.cn/szdw/dsdw/xyds/2023j1/687837de84704db9853f648c9febdf0c.htm</t>
+        </is>
+      </c>
+      <c r="R11" s="2" t="inlineStr">
+        <is>
+          <t>bit</t>
+        </is>
+      </c>
+      <c r="S11" s="2" t="inlineStr">
+        <is>
+          <t>北京理工大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>吕珍涛</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>education_background</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>博士后研究</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>海德堡大学</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr"/>
+      <c r="G12" s="2" t="inlineStr"/>
+      <c r="H12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr"/>
+      <c r="J12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="M12" s="2" t="inlineStr"/>
+      <c r="N12" s="2" t="inlineStr"/>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>本轮按留存来源记录整理；学位资格为来源记载，不代表独立证书认证。</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr"/>
+      <c r="Q12" s="3" t="inlineStr">
+        <is>
+          <t>https://qiushi.bit.edu.cn/szdw/dsdw/xyds/2023j1/687837de84704db9853f648c9febdf0c.htm</t>
+        </is>
+      </c>
+      <c r="R12" s="2" t="inlineStr">
+        <is>
+          <t>bit</t>
+        </is>
+      </c>
+      <c r="S12" s="2" t="inlineStr">
+        <is>
+          <t>北京理工大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>吕珍涛</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>employment</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr"/>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>北京理工大学</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr"/>
+      <c r="G13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr"/>
+      <c r="J13" s="2" t="inlineStr"/>
+      <c r="K13" s="2" t="inlineStr"/>
+      <c r="L13" s="2" t="inlineStr"/>
+      <c r="M13" s="2" t="inlineStr"/>
+      <c r="N13" s="2" t="inlineStr"/>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>任职按留存来源表述保留；不据此认证当前人事状态。；来源记载（单位）：数学与统计学院</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="inlineStr"/>
+      <c r="Q13" s="3" t="inlineStr">
+        <is>
+          <t>https://qiushi.bit.edu.cn/szdw/dsdw/xyds/2023j1/687837de84704db9853f648c9febdf0c.htm</t>
+        </is>
+      </c>
+      <c r="R13" s="2" t="inlineStr">
+        <is>
+          <t>bit</t>
+        </is>
+      </c>
+      <c r="S13" s="2" t="inlineStr">
+        <is>
+          <t>北京理工大学</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S8"/>
+  <autoFilter ref="A1:S13"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -1150,6 +1489,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q6" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q7" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q13" r:id="rId12"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1404,14 +1748,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="36.4" customWidth="1" min="2" max="2"/>
+    <col width="62.99999999999999" customWidth="1" min="2" max="2"/>
     <col width="65" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="65" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
@@ -1552,12 +1896,50 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>吕珍涛</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>new-recovery-bit-lyuzhentao-s001-14573b78be70</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>https://qiushi.bit.edu.cn/szdw/dsdw/xyds/2023j1/687837de84704db9853f648c9febdf0c.htm</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>留存来源记录（本轮重新审查；非独立证书认证）；NEW_RECOVERY：依据留存来源摘录、摘要或结构化记录；除另有本轮证据说明外未重新读取原网页，不继承旧核验结论。</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25T05:32:50Z</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>bit</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>北京理工大学</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G4"/>
+  <autoFilter ref="A1:G5"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>